<commit_message>
Se agrega LOGIN, proteccion de rutas al frontend, detalles de seguridad y funciones de edicion
</commit_message>
<xml_diff>
--- a/CHASIS HUB GUARENAS ACT.xlsx
+++ b/CHASIS HUB GUARENAS ACT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MissaelWave\Documents\Programacion\Proyectos\olt-dashboard-copia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B1677C-EABB-402E-9510-775F7C263E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0A0B13-42AA-439A-888F-143476583A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GRN-OLT1" sheetId="10" r:id="rId1"/>
@@ -5231,7 +5231,7 @@
   <dimension ref="A1:M113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" style="11" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="11" customWidth="1"/>
     <col min="3" max="3" width="9.28515625" style="11" customWidth="1"/>
     <col min="4" max="4" width="6.28515625" style="11" customWidth="1"/>
@@ -9753,10 +9753,10 @@
         <v>144</v>
       </c>
       <c r="H111" s="6">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I111" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J111" s="10">
         <v>7</v>

</xml_diff>